<commit_message>
Updated Sort and Filter.xlsx
</commit_message>
<xml_diff>
--- a/Sort and Filter.xlsx
+++ b/Sort and Filter.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Besant\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{72D024F2-E3BA-40D3-9132-A7D64E9ED822}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6486A29-F4BE-4328-AC5D-CCB4E5B03F09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{AAA77020-0F21-4DDF-B3BD-997AE361F6D3}"/>
   </bookViews>
@@ -336,168 +336,7 @@
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="16">
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -1919,7 +1758,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="X8:Y10" xr:uid="{25789103-A27A-4953-B83A-8AB05B2624B9}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="M2:S21">
     <sortCondition ref="M1:M21"/>
   </sortState>

</xml_diff>

<commit_message>
Improve Sort & Filter documentation
</commit_message>
<xml_diff>
--- a/Sort and Filter.xlsx
+++ b/Sort and Filter.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Besant\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6486A29-F4BE-4328-AC5D-CCB4E5B03F09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EEE016B-A144-4C37-B3A1-ECF79197D9FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{AAA77020-0F21-4DDF-B3BD-997AE361F6D3}"/>
   </bookViews>
@@ -23,21 +23,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="80">
   <si>
     <t>Employee Name</t>
   </si>
@@ -271,6 +262,12 @@
   </si>
   <si>
     <t>2. Training with west</t>
+  </si>
+  <si>
+    <t>this is a  OR structure.</t>
+  </si>
+  <si>
+    <t>this is a AND structure.</t>
   </si>
 </sst>
 </file>
@@ -1124,6 +1121,9 @@
       <c r="X9" t="s">
         <v>22</v>
       </c>
+      <c r="Z9" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="10" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A10">
@@ -1474,7 +1474,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="17" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>13</v>
       </c>
@@ -1525,8 +1525,11 @@
       <c r="Y17" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="18" spans="1:25" x14ac:dyDescent="0.35">
+      <c r="Z17" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="18" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>9</v>
       </c>
@@ -1575,7 +1578,7 @@
         <v>6250</v>
       </c>
     </row>
-    <row r="19" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>1</v>
       </c>
@@ -1624,7 +1627,7 @@
         <v>8750</v>
       </c>
     </row>
-    <row r="20" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>20</v>
       </c>
@@ -1673,7 +1676,7 @@
         <v>11250</v>
       </c>
     </row>
-    <row r="21" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>5</v>
       </c>
@@ -1719,7 +1722,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="28" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:26" x14ac:dyDescent="0.35">
       <c r="E28" t="s">
         <v>61</v>
       </c>
@@ -1727,22 +1730,22 @@
         <v>62</v>
       </c>
     </row>
-    <row r="29" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:26" x14ac:dyDescent="0.35">
       <c r="F29" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="30" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:26" x14ac:dyDescent="0.35">
       <c r="F30" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="31" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:26" x14ac:dyDescent="0.35">
       <c r="F31" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="32" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:26" x14ac:dyDescent="0.35">
       <c r="F32" t="s">
         <v>66</v>
       </c>

</xml_diff>